<commit_message>
Operatori Depureco (solo nome) e modalita demo della dashboard con 20 offerte fittizie
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/01_Matrice_Prezzi_Depureco.xlsx
+++ b/excel/01_Matrice_Prezzi_Depureco.xlsx
@@ -18578,7 +18578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -18613,19 +18613,65 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ufficio Commerciale Depureco</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>depureco@depureco.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>+39 011 9859117</t>
-        </is>
-      </c>
+          <t>Sabrina Menon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gianluca Prina</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Federico Pistone</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fabio Barberi</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mariacristina Rolle</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Marco Devincentis</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fabio Stura</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>